<commit_message>
feat(sizing): ~1h task sizing rule + backlog resize (R-005)
Skill SKILL.md gets a 'Task sizing rule' (size, club, split, clubbing-safe-pair
test, concrete heuristics); INTEGRATION.md mirrors it; deep-worker prompt picks
up NEEDS_SPLIT: PR slot and the 1-hour framing.

Backlog resized live via ledger ops: R1/R10/R11 SUPERSEDED -> R1a+R1b, R10a+R10b,
R11a+R11b; small winner-file reviews clubbed into TASK-R13 trio digest; size_hint
stamped on right-sized tasks. Ledger now 20 BACKLOG / 3 BLOCKED / 3 SUPERSEDED.
selector still picks owner(40); 93 tests green; dashboard regenerated.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T07:27:55.217347+00:00</t>
+          <t>2026-05-30T07:50:27.817191+00:00</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1116,6 +1116,266 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TASK-R1-category-taxonomy</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>SUPERSEDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>TASK-R1a-category-taxonomy-doc</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Category taxonomy + value ranking (doc only)</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>H-001</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>TASK-R1b-category-classifier</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rule classifier + tests for the taxonomy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>H-001</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TASK-R10-sft-training-kernel</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>SUPERSEDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>TASK-R10a-train-script-and-smoke</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TASK-R10b-kernel-metadata-readme</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TASK-R11-discussion-meta-analysis</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>SUPERSEDED</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TASK-R11a-discussion-do-avoid</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>H-007</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>H-007</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TASK-R13-winner-trio-digest</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>US-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(dispatcher): owner-role auto-dispatch + Wave-1 LIVE LAUNCH
dispatcher.dispatch_ready(): pick READY tasks (skip in-flight + blocked_by),
acquire per-area locks, render deep-worker prompt, create Jules sessions, atomic
ledger patch (record_session + set_status IN_PROGRESS + link). promote_backlog()
helper for the goal-loop. tools commands: dispatch, promote.

WAVE-1 LIVE (5 real Jules sessions IN_PROGRESS at jules.google):
- TASK-R1a category taxonomy doc       (sess 9152147452051460438)
- TASK-R10a train.py + smoke           (sess 3224516737148809732)
- TASK-R11a discussion do/avoid        (sess 18046708952198334024)
- TASK-R12 writeup skeleton            (sess 7801873606779501347)
- TASK-R13 winner trio digest          (sess 9044919978019878599)
Legacy US-* tasks SUPERSEDED (covered by R-tasks). 99 tests green.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T07:50:27.817191+00:00</t>
+          <t>2026-05-30T08:02:21.848357+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -580,7 +580,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -612,7 +612,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -740,7 +740,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -772,7 +772,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -804,7 +804,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -863,49 +863,24 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -915,145 +890,110 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>H-008</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>H-003</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1063,98 +1003,93 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>H-004</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>H-005</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>H-007</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1166,88 +1101,113 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-R13-winner-trio-digest</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1257,125 +1217,165 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>H-002</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-003</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R8</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>Local CV eval harness mirroring host scoring</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-004</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R9</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-005</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1605,6 +1605,91 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>18046708952198334024</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TASK-R11a-discussion-do-avoid</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>3224516737148809732</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TASK-R10a-train-script-and-smoke</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7801873606779501347</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TASK-R12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>9044919978019878599</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TASK-R13-winner-trio-digest</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>9152147452051460438</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TASK-R1a-category-taxonomy-doc</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tick RUN-20260530-083637: auto-merged 8 PRs, dispatched Wave-2 (5 sessions), seeded 4 hypotheses
- Auto-merged PRs #4 #5 #6 (orphan early-batch) + #7 #8 #9 #10 #11 (current
  batch) to main via force=True; all 8 R-007 unsupervised merges succeeded; 5
  tasks marked DONE.
- Promoted backlog (R1b/R10b/R11b unblocked by parent DONE; R7/R8/R9 already
  READY); superseded legacy stubs R1/R10/R11/R2.<cat>.
- Dispatched Wave-2 (cap=5 concurrent): TASK-K0 Kaggle smoke, R1b classifier,
  R7 CoT generator, R8 CV harness, R9 corpus curation (wait, dispatched were
  K0/R10b/R11b/R1b/R7 — selector picked oldest first); all IN_PROGRESS.
- Innovator: seeded H-DQ (data quality lever), H-LORA32 (winner config anchor,
  supported), H-1EPOCH, H-NORL; linked to in-flight tasks.
- Dashboard renderer hardened: list/dict cells coerced, openpyxl illegal-chars
  stripped (was crashing on \boxed{} in hypothesis text).
- 108 tests green.
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T08:02:21.848357+00:00</t>
+          <t>2026-05-30T08:50:44.175219+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -826,147 +826,147 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-OPS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-R1</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>H-001</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-R10</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -988,98 +988,98 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>H-007</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1101,12 +1101,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1116,81 +1116,81 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1202,17 +1202,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1234,64 +1234,59 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>H-003</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1301,79 +1296,116 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>H-004</t>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>TASK-R8</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Local CV eval harness mirroring host scoring</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>TASK-R9</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>READY</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>H-005</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>US-3</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G28" t="inlineStr">
         <is>
           <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
@@ -1390,7 +1422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1417,6 +1449,114 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>source_refs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>H-1EPOCH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1-epoch SFT is sufficient given high-quality CoT; more epochs over-fit on synthetic patterns.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>simpler training; no degradation</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>winner-train_sft.py.md, winner-loss_config.py.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>H-LORA32</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>matches winner; cheaper variants underperform</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>winner-train_sft.py.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>H-NORL</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>saves compute; lower risk</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>winner-INDEX.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
@@ -1580,7 +1720,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1608,12 +1748,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>18046708952198334024</t>
+          <t>14163923906156693592</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1625,12 +1765,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>3224516737148809732</t>
+          <t>15297474666584217295</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1642,12 +1782,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7801873606779501347</t>
+          <t>17312665199062602490</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1659,32 +1799,142 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9044919978019878599</t>
+          <t>18046708952198334024</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://github.com/manojdadi56/Kaggle/pull/10</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>18401029609494141683</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TASK-R7</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3224516737148809732</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TASK-R10a-train-script-and-smoke</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://github.com/manojdadi56/Kaggle/pull/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>7801873606779501347</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TASK-R12</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://github.com/manojdadi56/Kaggle/pull/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>9044919978019878599</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TASK-R13-winner-trio-digest</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://github.com/manojdadi56/Kaggle/pull/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>9152147452051460438</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://github.com/manojdadi56/Kaggle/pull/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9538569035955801003</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TASK-K0-kaggle-access-smoke</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>

</xml_diff>

<commit_message>
tick RUN-20260530-090133: auto-merged Wave-2 (PR #12 R11b deltas+hypotheses, #13 R7 CoT-gen), dispatched R8 R9, seeded 5 testable hypotheses (cipher/equation/bit-manip/curriculum/rank16) + 5 test tasks R20-R24
- Auto-merged PR #12 (R11b deltas+hypotheses) and PR #13 (R7 verified CoT-gen)
  via R-007 unsupervised path; tasks set DONE; 7 stale-completed sessions
  cleared from state.
- 5 jules sessions in flight now: K0 R1b R10b R8 R9.
- Innovator: appended H-CIPHER-100 / H-EQ-SYMPY / H-BIT-NICKNAME (per-category
  solvable in cited threads), H-CURRICULUM (difficulty ordering), H-RANK16
  (compute-efficient ablation). Linked corresponding deep tasks R20..R24
  (~45-75 min each per R-005). BACKLOG = 5 next-up tests.
- Hypotheses total 9; tasks 32; dashboard refreshed.
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T08:50:44.175219+00:00</t>
+          <t>2026-05-30T09:05:52.079556+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1303,109 +1303,269 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>US-2</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>TASK-R22-bit-manipulation-solver</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>H-BIT-NICKNAME</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TASK-R23-curriculum-config</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>H-CURRICULUM</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>TASK-R24-rank16-ablation-kernel</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>H-RANK16</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>TASK-R7</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>TASK-R8</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Local CV eval harness mirroring host scoring</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
           <t>TASK-R9</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
         <is>
           <t>H-DQ</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>US-3</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
+      <c r="G33" t="inlineStr">
         <is>
           <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
@@ -1422,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1482,12 +1642,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
+          <t>Bit-manipulation problems use nickname encodings (e.g. "the integer formed by bytes…"); a robust regex extractor across all 1602 bit_manipulation rows yields 100% solver coverage.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1497,66 +1657,201 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
+          <t>+0.17 LB on bit_manipulation category</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
+          <t>winner-reasoning.py.md, discussion-689915.md</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+          <t>Cipher-category problems reduce to substitution+offset and admit a 100% deterministic solver.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>matches winner; cheaper variants underperform</t>
+          <t>+0.16 LB from solving all 1576 cipher rows in train + matching test distribution</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md</t>
+          <t>winner-reasoning.py.md, discussion-689915.md</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>H-CURRICULUM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Difficulty-ordered curriculum SFT (easy→hard within each category) generalizes better than random shuffle on the hidden test set.</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>+0.01-0.03 LB vs random ordering, free improvement</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>discussion-688360.md, DIGEST-community.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>H-EQ-SYMPY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Equation-numeric problems are solvable with SymPy linear/quadratic solvers; algebraic CoT is reproducible.</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>+0.07 LB on equation_numeric_deduce(596)+_guess(136) categories</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, technique-backlog.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>H-LORA32</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>matches winner; cheaper variants underperform</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>winner-train_sft.py.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>H-NORL</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>saves compute; lower risk</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>winner-INDEX.md, DIGEST-community.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>H-RANK16</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>~equal LB, 2x cheaper experiments</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
@@ -1720,7 +2015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1748,46 +2043,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>14163923906156693592</t>
+          <t>15297474666584217295</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>15297474666584217295</t>
+          <t>17312665199062602490</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>17312665199062602490</t>
+          <t>3615961847482794211</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R9</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1799,144 +2094,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>18046708952198334024</t>
+          <t>8303277900745917951</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R8</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>https://github.com/manojdadi56/Kaggle/pull/10</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>18401029609494141683</t>
+          <t>9538569035955801003</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3224516737148809732</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://github.com/manojdadi56/Kaggle/pull/11</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>7801873606779501347</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TASK-R12</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>https://github.com/manojdadi56/Kaggle/pull/9</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>9044919978019878599</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>TASK-R13-winner-trio-digest</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>https://github.com/manojdadi56/Kaggle/pull/7</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>9152147452051460438</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>https://github.com/manojdadi56/Kaggle/pull/8</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>9538569035955801003</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-114605: E-002 still in flight; E-007 steered (achieved 100% classifier coverage)
Nothing terminalized this tick. E-002 baseline still IN_PROGRESS (kernel
authoring is heavier than solver authoring). E-007 came back with significant
progress — the classify.py fix differentiating equation_numeric vs cryptarithm
now covers 100 percent of train. Steered to proceed with the remaining 3 task
steps and ship the PR.

2 in flight (E-002, E-007). 6 BLOCKED ablation children correctly waiting
on E-002 by design. Selector picks planner but no actionable backlog (the
chain is correct, not stuck).

Note: build_corpus.py requires transformers + Nemotron tokenizer download
(non-trivial setup) — local validation of the corpus output deferred to
when E-002 kernel runs on Kaggle GPU which has the dependencies cached.

Ledger: 18 hypotheses, 10 experiments, 47 tasks (24 DONE / 2 IN_PROGRESS /
6 BLOCKED / 0 READY / 15 SUPERSEDED). 115 tests still green.
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T11:18:15.860341+00:00</t>
+          <t>2026-05-30T11:46:39.064262+00:00</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3063,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>AWAITING_USER_FEEDBACK</t>
         </is>
       </c>
     </row>
@@ -3080,7 +3080,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-114605b: dashboard + reporter log (planner appended H-VLLM-EVAL/H-SUBMIT-GATE)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T11:46:39.064262+00:00</t>
+          <t>2026-05-30T12:16:42.181093+00:00</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1146,174 +1146,164 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>US-OPS</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-OPS</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-R1</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>H-001</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-R10</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1323,12 +1313,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1340,93 +1330,93 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R11</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>H-007</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1441,7 +1431,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1453,12 +1443,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1468,34 +1458,29 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1505,29 +1490,34 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1537,12 +1527,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1554,12 +1544,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1574,7 +1564,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1586,81 +1576,81 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>US-3</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1670,12 +1660,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1687,12 +1677,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1702,12 +1692,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1719,12 +1709,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1734,12 +1724,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1751,12 +1741,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1766,29 +1756,29 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1798,29 +1788,29 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1830,12 +1820,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1847,12 +1837,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1862,12 +1852,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1879,12 +1869,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1894,12 +1884,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1911,12 +1901,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1926,29 +1916,29 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R29-eval-per-category-breakdown</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1963,29 +1953,24 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+          <t>US-2</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2000,54 +1985,113 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>TASK-R8</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Local CV eval harness mirroring host scoring</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>TASK-R9</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>H-DQ</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>US-3</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G49" t="inlineStr">
         <is>
           <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-validate-adapter</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2554,27 +2598,81 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>H-SUBMIT-GATE</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>H-UNIT-CONV-100</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>proposed</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>+0.17 LB on 1594 unit_conversion rows</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>H-VLLM-EVAL</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3161,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AWAITING_USER_FEEDBACK</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-114605c: dashboard + reporter log (pipeline-completion: train/validate/submit)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T12:16:42.181093+00:00</t>
+          <t>2026-05-30T12:22:27.657986+00:00</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1146,12 +1146,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-EVAL-cv-fixture</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
+          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1161,213 +1161,188 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-EVAL-cv-score-ingest</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>US-OPS</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>H-001</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>H-OPS</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>H-006</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-OPS-run-kernel-runner</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-R1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>H-LORA32</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1377,29 +1352,29 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1411,12 +1386,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1426,29 +1401,29 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1458,98 +1433,78 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>US-6</t>
+          <t>US-1</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1559,12 +1514,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -1576,12 +1531,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1591,12 +1546,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -1608,49 +1563,49 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-6</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1660,29 +1615,29 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1692,29 +1647,29 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1724,61 +1679,66 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>US-3</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1788,29 +1748,29 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1820,12 +1780,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1837,12 +1797,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1852,12 +1812,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1869,12 +1829,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1884,12 +1844,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1901,12 +1861,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1916,29 +1876,29 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1948,29 +1908,29 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1980,34 +1940,29 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2017,34 +1972,29 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>US-2</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2054,42 +2004,224 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>TASK-R29-eval-per-category-breakdown</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>TASK-R7</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>TASK-R8</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Local CV eval harness mirroring host scoring</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>TASK-R9</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-gate-decision</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-package-zip</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>TASK-SUBMIT-validate-adapter</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
         </is>
@@ -2106,7 +2238,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2382,39 +2514,39 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-GPU-DISPATCH</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
+          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
+          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
+          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2424,78 +2556,78 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+0.01 LB on hard categories.</t>
+          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-LOGPROB-FILTER</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>matches winner; cheaper variants underperform</t>
+          <t>+0.01 LB on hard categories.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md</t>
+          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>H-MAMBA-TARGETS</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>supported</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Unblocks training on free GPU. Critical precondition.</t>
+          <t>matches winner; cheaper variants underperform</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, multiple discussions</t>
+          <t>winner-train_sft.py.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>H-NORL</t>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
+          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2505,24 +2637,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>saves compute; lower risk</t>
+          <t>Unblocks training on free GPU. Critical precondition.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md</t>
+          <t>analysis-discussions-deltas.md, multiple discussions</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-NORL</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
+          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2532,24 +2664,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+0.16 LB on 1576 numeral rows</t>
+          <t>saves compute; lower risk</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2559,24 +2691,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>~equal LB, 2x cheaper experiments</t>
+          <t>+0.16 LB on 1576 numeral rows</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md, technique-backlog.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2586,91 +2718,118 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>~equal LB at half cost; may slightly improve generalization.</t>
+          <t>~equal LB, 2x cheaper experiments</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>H-SUBMIT-GATE</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+          <t>~equal LB at half cost; may slightly improve generalization.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-SUBMIT-GATE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>+0.17 LB on 1594 unit_conversion rows</t>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>H-UNIT-CONV-100</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>+0.17 LB on 1594 unit_conversion rows</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>H-VLLM-EVAL</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>

</xml_diff>

<commit_message>
tick RUN-20260530-122402: E-002 merged + large fanout dispatch (9 parallel: 5 ablations + 4 pipeline)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T12:22:27.657986+00:00</t>
+          <t>2026-05-30T12:26:44.730251+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
@@ -900,7 +900,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3282,7 +3282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3310,34 +3310,170 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13107147469450254389</t>
+          <t>13013155406031425658</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>5869851881805383251</t>
+          <t>13107147469450254389</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-E002-baseline-kernel</t>
+          <t>TASK-E007-cryptarithm-guess-integration</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>IN_PROGRESS</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>14674823960857717074</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TASK-E003-rank16-finalize</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>14769124856858592956</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TASK-E004-2epoch-kernel</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>3331869219988151080</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TASK-E006-select2reason</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5459254010184172264</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TASK-E005-curriculum-wire</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6684794983844118444</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TASK-OPS-run-kernel-runner</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>728421577080239025</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TASK-E008-logprob-filter</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8195905385648107214</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>TASK-EVAL-cv-fixture</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>9916984275388767522</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-validate-adapter</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-124519: 8 PRs merged (#32-#39); gpu-dispatch + package-zip dispatched
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T12:26:44.730251+00:00</t>
+          <t>2026-05-30T12:48:24.531044+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -932,7 +932,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -964,7 +964,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -996,7 +996,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1200,7 +1200,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2218,7 +2218,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -3282,7 +3282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3310,46 +3310,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13013155406031425658</t>
+          <t>13107147469450254389</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-E007-cryptarithm-guess-integration</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13107147469450254389</t>
+          <t>15457649004442238545</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>14674823960857717074</t>
+          <t>290296703496810863</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TASK-E003-rank16-finalize</t>
+          <t>TASK-SUBMIT-package-zip</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3361,119 +3361,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>14769124856858592956</t>
+          <t>728421577080239025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TASK-E004-2epoch-kernel</t>
+          <t>TASK-E008-logprob-filter</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>3331869219988151080</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>TASK-E006-select2reason</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5459254010184172264</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TASK-E005-curriculum-wire</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>6684794983844118444</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TASK-OPS-run-kernel-runner</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>728421577080239025</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>TASK-E008-logprob-filter</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>8195905385648107214</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>TASK-EVAL-cv-fixture</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>9916984275388767522</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>TASK-SUBMIT-validate-adapter</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-131519: #40+#41 merged; package-zip rescued operator-side; 3 final-chain tasks dispatched
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T12:48:24.531044+00:00</t>
+          <t>2026-05-30T13:21:30.026016+00:00</t>
         </is>
       </c>
     </row>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1254,7 +1254,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -3310,46 +3310,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>13107147469450254389</t>
+          <t>11172407645040114728</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-E009-synthesis-kernel</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>15457649004442238545</t>
+          <t>13107147469450254389</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-OPS-gpu-dispatch-op</t>
+          <t>TASK-E007-cryptarithm-guess-integration</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>290296703496810863</t>
+          <t>15996892913727706506</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-package-zip</t>
+          <t>TASK-SUBMIT-gate-decision</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3361,17 +3361,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>728421577080239025</t>
+          <t>5860122008944918375</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TASK-E008-logprob-filter</t>
+          <t>TASK-EVAL-cv-score-ingest</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-134333: planner: H-AUTO-RESCUE + H-CHAT-TEMPLATE; E-009 steered
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T13:21:30.026016+00:00</t>
+          <t>2026-05-30T13:48:44.735123+00:00</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1146,78 +1146,78 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-fixture</t>
+          <t>TASK-EVAL-chat-template-parity</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
+          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-score-ingest</t>
+          <t>TASK-EVAL-cv-fixture</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
+          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-EVAL-cv-score-ingest</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
+          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1225,31 +1225,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
-        </is>
-      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>US-OPS</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-OPS-gpu-dispatch-op</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1257,92 +1247,97 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>H-OPS</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-OPS-run-kernel-runner</t>
+          <t>TASK-OPS-auto-rescue</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
+          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
+          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>H-001</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-OPS-run-kernel-runner</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
+          <t>TASK-R1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1352,29 +1347,29 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1386,17 +1381,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-R10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1406,110 +1401,110 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>US-4</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>H-LORA32</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>H-LORA32</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R11</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1519,56 +1514,41 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>US-1</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1578,34 +1558,29 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1615,12 +1590,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1632,12 +1607,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1647,29 +1622,34 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1679,12 +1659,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1696,49 +1676,44 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1748,61 +1723,66 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>US-3</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1812,12 +1792,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1829,12 +1809,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1844,12 +1824,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1861,12 +1841,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1876,29 +1856,29 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1908,12 +1888,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1925,12 +1905,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1940,29 +1920,29 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1972,12 +1952,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -1989,12 +1969,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2004,12 +1984,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2021,12 +2001,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2036,29 +2016,29 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2068,34 +2048,29 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R29-eval-per-category-breakdown</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2116,23 +2091,18 @@
       <c r="F52" t="inlineStr">
         <is>
           <t>US-2</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2147,7 +2117,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2157,41 +2127,56 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-gate-decision</t>
+          <t>TASK-R8</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+          <t>Local CV eval harness mirroring host scoring</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-package-zip</t>
+          <t>TASK-R9</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2199,29 +2184,88 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
+          <t>TASK-SUBMIT-gate-decision</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-package-zip</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>TASK-SUBMIT-validate-adapter</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
         </is>
@@ -2238,7 +2282,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2298,39 +2342,39 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-AUTO-RESCUE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bit-manipulation problems use nickname encodings (e.g. "the integer formed by bytes…"); a robust regex extractor across all 1602 bit_manipulation rows yields 100% solver coverage.</t>
+          <t>Tick RUN-20260530-131519 surfaced a real failure mode: session 290296703496810863 emitted sessionCompleted with a complete unidiff in its artifact (tools/package_submission.py + tests/test_package_submission.py) but never opened a GitHub PR. The operator had to manually extract the patch, apply it to a rescue branch, run pytest, and merge to main. Adding an operator-side auto-rescue path inside orchestrator/loop.py.poll_in_flight - when a session returns state=COMPLETED with pr_url=None, fetch /sessions/&lt;sid&gt;/activities, find the last sessionCompleted artifact gitPatch, apply it to a fresh branch, run pytest -q, merge to main via the existing R-007 force-merge path - eliminates this whole manual step.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>+0.17 LB on bit_manipulation category</t>
+          <t>Removes one human-in-the-loop step per failure. Observed rate: 1/11 dispatches in the RUN-20260530-124519 fanout. At scale (50-100 sessions/day expected near deadline), this saves ~5-10 manual rescues/day.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, discussion-689915.md</t>
+          <t>state/run_log.jsonl tick RUN-20260530-131519, orchestrator/loop.py poll_in_flight, orchestrator/github_ops.py merge_pr</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cipher-category problems reduce to substitution+offset and admit a 100% deterministic solver.</t>
+          <t>Bit-manipulation problems use nickname encodings (e.g. "the integer formed by bytes…"); a robust regex extractor across all 1602 bit_manipulation rows yields 100% solver coverage.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2340,7 +2384,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>+0.16 LB from solving all 1576 cipher rows in train + matching test distribution</t>
+          <t>+0.17 LB on bit_manipulation category</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2352,39 +2396,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-CHAT-TEMPLATE</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce problems are uniquely solvable letter-digit assignment problems; constraint propagation (or python-constraint / Z3) yields the exact answer.</t>
+          <t>Discussions repeatedly note that the host scoring runs inference with a SPECIFIC chat template (Nemotron-3-Nano-30B-A3B-BF16 default + reasoning_on header). If our LoRA adapter is trained or evaluated under a different template (e.g. our eval/vllm_eval.py uses ChatML where host uses Nemotron's native), every output is a few tokens off and \boxed{} extraction may miss. Adding eval/test_chat_template_parity.py that loads the official tokenizer's apply_chat_template on a known fixture and asserts byte-equality vs the harness's rendered prompt prevents this.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>+0.07 LB on 659+164 cryptarithm rows</t>
+          <t>Catches a class of silent failures that would only manifest as 'CV looks 0.0 on a well-trained adapter' - very hard to debug after the fact.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>discussion-682208.md, discussion-690161.md, winner-train_sft.py.md (chat template usage), tab-rules.md (host scoring spec)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM-GUESS</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Winner skipped cryptarithm_guess; adding a solver + verified CoT for it gives direct LB headroom (164 train rows).</t>
+          <t>Cipher-category problems reduce to substitution+offset and admit a 100% deterministic solver.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2394,24 +2438,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>+0.01-0.03 LB direct from a category the winner never trained on.</t>
+          <t>+0.16 LB from solving all 1576 cipher rows in train + matching test distribution</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-reasoning.py.md</t>
+          <t>winner-reasoning.py.md, discussion-689915.md</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Difficulty-ordered curriculum SFT (easy→hard within each category) generalizes better than random shuffle on the hidden test set.</t>
+          <t>Cryptarithm-deduce problems are uniquely solvable letter-digit assignment problems; constraint propagation (or python-constraint / Z3) yields the exact answer.</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2421,24 +2465,24 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>+0.01-0.03 LB vs random ordering, free improvement</t>
+          <t>+0.07 LB on 659+164 cryptarithm rows</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>discussion-688360.md, DIGEST-community.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM-GUESS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
+          <t>Winner skipped cryptarithm_guess; adding a solver + verified CoT for it gives direct LB headroom (164 train rows).</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2448,24 +2492,24 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
+          <t>+0.01-0.03 LB direct from a category the winner never trained on.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
+          <t>analysis-discussions-deltas.md, winner-reasoning.py.md</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>H-EQ-FALLBACK</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Default to absolute-difference fallback in equation_numeric solvers when no rule is found; captures edge cases.</t>
+          <t>Difficulty-ordered curriculum SFT (easy→hard within each category) generalizes better than random shuffle on the hidden test set.</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2475,24 +2519,24 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>+0.01 LB on equation_numeric category.</t>
+          <t>+0.01-0.03 LB vs random ordering, free improvement</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-reasoning.py.md</t>
+          <t>discussion-688360.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Equation-numeric problems are solvable with SymPy linear/quadratic solvers; algebraic CoT is reproducible.</t>
+          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2502,51 +2546,51 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+0.07 LB on equation_numeric_deduce(596)+_guess(136) categories</t>
+          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, technique-backlog.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>H-GPU-DISPATCH</t>
+          <t>H-EQ-FALLBACK</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
+          <t>Default to absolute-difference fallback in equation_numeric solvers when no rule is found; captures edge cases.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
+          <t>+0.01 LB on equation_numeric category.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
+          <t>analysis-discussions-deltas.md, winner-reasoning.py.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
+          <t>Equation-numeric problems are solvable with SymPy linear/quadratic solvers; algebraic CoT is reproducible.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2556,78 +2600,78 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
+          <t>+0.07 LB on equation_numeric_deduce(596)+_guess(136) categories</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>winner-reasoning.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-GPU-DISPATCH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
+          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>+0.01 LB on hard categories.</t>
+          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
+          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>matches winner; cheaper variants underperform</t>
+          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>H-MAMBA-TARGETS</t>
+          <t>H-LOGPROB-FILTER</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
+          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2637,51 +2681,51 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Unblocks training on free GPU. Critical precondition.</t>
+          <t>+0.01 LB on hard categories.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, multiple discussions</t>
+          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>H-NORL</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>supported</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>saves compute; lower risk</t>
+          <t>matches winner; cheaper variants underperform</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md</t>
+          <t>winner-train_sft.py.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
+          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2691,24 +2735,24 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+0.16 LB on 1576 numeral rows</t>
+          <t>Unblocks training on free GPU. Critical precondition.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>analysis-discussions-deltas.md, multiple discussions</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-NORL</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2718,24 +2762,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>~equal LB, 2x cheaper experiments</t>
+          <t>saves compute; lower risk</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md, technique-backlog.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
+          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2745,51 +2789,51 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>~equal LB at half cost; may slightly improve generalization.</t>
+          <t>+0.16 LB on 1576 numeral rows</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H-SUBMIT-GATE</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>proposed</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+          <t>~equal LB, 2x cheaper experiments</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2799,37 +2843,91 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>+0.17 LB on 1594 unit_conversion rows</t>
+          <t>~equal LB at half cost; may slightly improve generalization.</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>H-SUBMIT-GATE</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>H-UNIT-CONV-100</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>proposed</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>+0.17 LB on 1594 unit_conversion rows</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>H-VLLM-EVAL</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>
@@ -3320,7 +3418,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3452,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3469,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>QUEUED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-135009: PR #43 merged; E-007 operator-rescued; auto-rescue + chat-template tasks dispatched
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T13:48:44.735123+00:00</t>
+          <t>2026-05-30T13:56:09.037696+00:00</t>
         </is>
       </c>
     </row>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1156,7 +1156,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1276,7 +1276,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3408,29 +3408,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11172407645040114728</t>
+          <t>11091484301140930622</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-E009-synthesis-kernel</t>
+          <t>TASK-EVAL-chat-template-parity</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>13107147469450254389</t>
+          <t>11172407645040114728</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-E009-synthesis-kernel</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3442,17 +3442,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>15996892913727706506</t>
+          <t>4390025997776432846</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-gate-decision</t>
+          <t>TASK-OPS-auto-rescue</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>QUEUED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tick RUN-20260530-141526: clear 3 COMPLETED sessions (PRs #44/#45/#46 auto-merged)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T13:56:09.037696+00:00</t>
+          <t>2026-05-30T14:01:18.959938+00:00</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G58"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -890,27 +890,22 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TASK-E002-baseline-kernel</t>
+          <t>TASK-E002-SMOKE-RUN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Finalize winner-faithful baseline training kernel (rank32/alpha64/1-epoch/LinearDecay)</t>
+          <t>Kaggle GPU smoke run: 5-min rank=4 max_steps=20 100-row preflight</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>H-LORA32</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -922,12 +917,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TASK-E003-rank16-finalize</t>
+          <t>TASK-E002-baseline-kernel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Align rank-16 ablation kernel (R24) with the E-002 config except rank/alpha</t>
+          <t>Finalize winner-faithful baseline training kernel (rank32/alpha64/1-epoch/LinearDecay)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -937,12 +932,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -954,27 +949,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TASK-E004-2epoch-kernel</t>
+          <t>TASK-E002-push-and-train</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Clone baseline kernel with epochs=2 (refutation test for H-1EPOCH)</t>
+          <t>Push baseline E-002 (rank=32) kernel to Kaggle GPU and ingest cv_score</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>H-1EPOCH</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-2epoch-e004</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -986,12 +976,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TASK-E005-curriculum-wire</t>
+          <t>TASK-E003-rank16-finalize</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Wire R23 curriculum config into the baseline kernel (difficulty-ascending)</t>
+          <t>Align rank-16 ablation kernel (R24) with the E-002 config except rank/alpha</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1001,12 +991,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-curriculum-e005</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1018,12 +1008,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TASK-E006-select2reason</t>
+          <t>TASK-E004-2epoch-kernel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Select2Reason curation: keep top-utility ~30 percent of corpus, then train baseline</t>
+          <t>Clone baseline kernel with epochs=2 (refutation test for H-1EPOCH)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1033,12 +1023,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-1EPOCH</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-select2reason-e006</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-2epoch-e004</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1050,12 +1040,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-E005-curriculum-wire</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Integrate cryptarithm_guess solver into corpus (winner skipped this category) — priority</t>
+          <t>Wire R23 curriculum config into the baseline kernel (difficulty-ascending)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1065,29 +1055,29 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM-GUESS</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-curriculum-e005</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TASK-E008-logprob-filter</t>
+          <t>TASK-E006-select2reason</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Pre-filter corpus by base-model min log-prob (drop already-easy examples)</t>
+          <t>Select2Reason curation: keep top-utility ~30 percent of corpus, then train baseline</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1097,12 +1087,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-logprob-filter-e008</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-select2reason-e006</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1114,66 +1104,71 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TASK-E009-synthesis-kernel</t>
+          <t>TASK-E007-RESCOPE</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Synthesis: combine winning ablation choices into final config</t>
+          <t>Rescope or abort stuck E-007 cryptarithm-guess Jules session</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>H-DQ</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-synthesis-e009</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/v1, competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm, competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-EVAL-chat-template-parity</t>
+          <t>TASK-E007-cryptarithm-guess-integration</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
+          <t>Integrate cryptarithm_guess solver into corpus (winner skipped this category) — priority</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>H-CRYPTARITHM-GUESS</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-fixture</t>
+          <t>TASK-E008-logprob-filter</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
+          <t>Pre-filter corpus by base-model min log-prob (drop already-easy examples)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1181,21 +1176,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>H-LOGPROB-FILTER</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-logprob-filter-e008</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-score-ingest</t>
+          <t>TASK-E009-synthesis-kernel</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
+          <t>Synthesis: combine winning ablation choices into final config</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1203,43 +1208,53 @@
           <t>IN_PROGRESS</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-synthesis-e009</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-EVAL-chat-template-parity</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
+          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-EVAL-cv-fixture</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1247,31 +1262,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
-        </is>
-      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>US-OPS</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-OPS-auto-rescue</t>
+          <t>TASK-EVAL-cv-score-ingest</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
+          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1281,19 +1286,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-OPS-gpu-dispatch-op</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1303,139 +1308,149 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-OPS-run-kernel-runner</t>
+          <t>TASK-FIX-kernel-metadata</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
+          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-OPS</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-OPS-auto-rescue</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
+          <t>TASK-OPS-cron-trigger</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>H-006</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+          <t>(scheduler only)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>US-meta</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-OPS-run-kernel-runner</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1443,144 +1458,119 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-R1</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R10</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1590,29 +1580,29 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1622,98 +1612,78 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R11</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>US-1</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>H-001</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1723,12 +1693,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -1740,49 +1710,44 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1792,29 +1757,34 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1824,29 +1794,29 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1856,29 +1826,29 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1888,61 +1858,66 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1952,12 +1927,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -1969,12 +1944,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1984,12 +1959,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2001,12 +1976,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2016,12 +1991,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2033,12 +2008,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2048,12 +2023,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2065,12 +2040,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2080,29 +2055,29 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2112,34 +2087,29 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2149,34 +2119,29 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>US-2</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2186,56 +2151,61 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-gate-decision</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-package-zip</t>
+          <t>TASK-R29-eval-per-category-breakdown</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2243,29 +2213,194 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>US-2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>TASK-R7</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>TASK-R8</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Local CV eval harness mirroring host scoring</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>TASK-R9</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-gate-decision</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-package-zip</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
           <t>TASK-SUBMIT-validate-adapter</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B63" t="inlineStr">
         <is>
           <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
         </is>
@@ -2325,7 +2460,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -2379,7 +2514,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -2433,7 +2568,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -2460,7 +2595,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -2487,7 +2622,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -2514,7 +2649,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -2541,7 +2676,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2568,7 +2703,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2595,7 +2730,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2649,7 +2784,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2676,7 +2811,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2703,7 +2838,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2730,7 +2865,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2757,7 +2892,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2784,7 +2919,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2811,7 +2946,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2838,7 +2973,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2892,7 +3027,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>proposed</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -3296,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3319,15 +3454,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>D-AUDIT-2026-05-30</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Pause new feature work; land the 6 audit-corrections + 5 seeded tasks before adding capability.</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Audit found 5 live defects (3 fixed mid-pass), 6 invalidated assumptions, 0 end-to-end runs. Infrastructure-complete but execution-untriggered. Adding features now compounds cross-PR invariant drift the audit identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>D-EXPLAN-001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Lock experimentation plan (Phase A done, B-&gt;C-&gt;D-&gt;E-&gt;F; E-007 cryptarithm_guess prioritized).</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Cross-validated against winner repo (R13), discussion deltas (R11b), 18 ledger hypotheses. See EXPERIMENTATION_PLAN.md.</t>
         </is>

</xml_diff>

<commit_message>
tick RUN-20260530-141526: PRs #44/#45/#46 merged; FIX-kernel-metadata dispatched (critical-path before first GPU)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T14:01:18.959938+00:00</t>
+          <t>2026-05-30T14:19:13.070627+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1205,7 +1205,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3532,7 +3532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3560,12 +3560,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>11091484301140930622</t>
+          <t>12749140667475037666</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>TASK-EVAL-chat-template-parity</t>
+          <t>TASK-FIX-kernel-metadata</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3577,49 +3577,15 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>11172407645040114728</t>
+          <t>4390025997776432846</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-E009-synthesis-kernel</t>
+          <t>TASK-OPS-auto-rescue</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>4390025997776432846</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>TASK-OPS-auto-rescue</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>5860122008944918375</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>TASK-EVAL-cv-score-ingest</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
         <is>
           <t>IN_PROGRESS</t>
         </is>

</xml_diff>

<commit_message>
tick RUN-20260530-150539: auto-rescue operator-merged; FIX-kernel-metadata steered to inline corpus build
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T14:19:13.070627+00:00</t>
+          <t>2026-05-30T15:13:55.362085+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -1384,7 +1384,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -3532,7 +3532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3570,23 +3570,6 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>4390025997776432846</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>TASK-OPS-auto-rescue</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
           <t>IN_PROGRESS</t>
         </is>
       </c>

</xml_diff>

<commit_message>
tick RUN-20260530-151543: watch mode; cron-trigger SUPERSEDED; FIX-kernel-metadata still authoring
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T15:13:55.362085+00:00</t>
+          <t>2026-05-30T15:18:10.643686+00:00</t>
         </is>
       </c>
     </row>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">

</xml_diff>

<commit_message>
tick RUN-20260530-155344: PR #47 merged (-X ours for live E-002); v4/v5/v6 GPU iteration (mamba-ssm pip install + diagnostics)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T15:18:10.643686+00:00</t>
+          <t>2026-05-30T16:17:49.352564+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -900,7 +900,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>READY</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3532,7 +3532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3557,23 +3557,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>12749140667475037666</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TASK-FIX-kernel-metadata</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
tick RUN-20260530-175941: P100 still blocking; SMOKE-RUN superseded; kaggle MCP registered (needs restart)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T16:17:49.352564+00:00</t>
+          <t>2026-05-30T18:02:44.546965+00:00</t>
         </is>
       </c>
     </row>
@@ -900,7 +900,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>READY</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">

</xml_diff>

<commit_message>
queue V15: CoT corpus inline patch (91 examples gz+b64=39KB); ready to fire after first submission
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T20:45:26.956597+00:00</t>
+          <t>2026-05-30T21:02:55.955233+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>62</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -826,44 +826,34 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TASK-E-PRECOND-mamba-targets-smoke</t>
+          <t>TASK-DATA-cot-corpus-v1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Smoke-train kernel (10 steps) validating Mamba mixer LoRA targeting</t>
+          <t>Build CoT corpus from train.csv using winner's deterministic solver pattern (the 0.65-&gt;0.85 lever)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>H-MAMBA-TARGETS</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/, tests/test_cot_corpus_v1.py</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TASK-E001-corpus-v1</t>
+          <t>TASK-E-PRECOND-mamba-targets-smoke</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Assemble corpus.jsonl v1 from landed solvers (winner build_datum convention)</t>
+          <t>Smoke-train kernel (10 steps) validating Mamba mixer LoRA targeting</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -873,71 +863,71 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TASK-E002-SMOKE-RUN</t>
+          <t>TASK-E001-corpus-v1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Kaggle GPU smoke run: 5-min rank=4 max_steps=20 100-row preflight</t>
+          <t>Assemble corpus.jsonl v1 from landed solvers (winner build_datum convention)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TASK-E002-baseline-kernel</t>
+          <t>TASK-E002-SMOKE-RUN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Finalize winner-faithful baseline training kernel (rank32/alpha64/1-epoch/LinearDecay)</t>
+          <t>Kaggle GPU smoke run: 5-min rank=4 max_steps=20 100-row preflight</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>H-LORA32</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -949,17 +939,22 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TASK-E002-push-and-train</t>
+          <t>TASK-E002-baseline-kernel</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Push baseline E-002 (rank=32) kernel to Kaggle GPU and ingest cv_score</t>
+          <t>Finalize winner-faithful baseline training kernel (rank32/alpha64/1-epoch/LinearDecay)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -976,27 +971,22 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TASK-E003-rank16-finalize</t>
+          <t>TASK-E002-push-and-train</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Align rank-16 ablation kernel (R24) with the E-002 config except rank/alpha</t>
+          <t>Push baseline E-002 (rank=32) kernel to Kaggle GPU and ingest cv_score</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>H-RANK16</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1008,12 +998,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TASK-E004-2epoch-kernel</t>
+          <t>TASK-E003-rank16-finalize</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Clone baseline kernel with epochs=2 (refutation test for H-1EPOCH)</t>
+          <t>Align rank-16 ablation kernel (R24) with the E-002 config except rank/alpha</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1023,12 +1013,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>H-1EPOCH</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-2epoch-e004</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1040,12 +1030,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TASK-E005-curriculum-wire</t>
+          <t>TASK-E004-2epoch-kernel</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Wire R23 curriculum config into the baseline kernel (difficulty-ascending)</t>
+          <t>Clone baseline kernel with epochs=2 (refutation test for H-1EPOCH)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1055,12 +1045,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-1EPOCH</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-curriculum-e005</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-2epoch-e004</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1072,12 +1062,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TASK-E006-select2reason</t>
+          <t>TASK-E005-curriculum-wire</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Select2Reason curation: keep top-utility ~30 percent of corpus, then train baseline</t>
+          <t>Wire R23 curriculum config into the baseline kernel (difficulty-ascending)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1087,12 +1077,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-select2reason-e006</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-curriculum-e005</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1104,12 +1094,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TASK-E007-RESCOPE</t>
+          <t>TASK-E006-select2reason</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Rescope or abort stuck E-007 cryptarithm-guess Jules session</t>
+          <t>Select2Reason curation: keep top-utility ~30 percent of corpus, then train baseline</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1117,26 +1107,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>H-SELECT2REASON</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/v1, competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm, competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-select2reason-e006</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-E007-RESCOPE</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Integrate cryptarithm_guess solver into corpus (winner skipped this category) — priority</t>
+          <t>Rescope or abort stuck E-007 cryptarithm-guess Jules session</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1144,14 +1139,9 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>H-CRYPTARITHM-GUESS</t>
-        </is>
-      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/v1, competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm, competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1163,12 +1153,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-E008-logprob-filter</t>
+          <t>TASK-E007-cryptarithm-guess-integration</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Pre-filter corpus by base-model min log-prob (drop already-easy examples)</t>
+          <t>Integrate cryptarithm_guess solver into corpus (winner skipped this category) — priority</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1178,29 +1168,29 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-CRYPTARITHM-GUESS</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-logprob-filter-e008</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-E009-synthesis-kernel</t>
+          <t>TASK-E008-logprob-filter</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Synthesis: combine winning ablation choices into final config</t>
+          <t>Pre-filter corpus by base-model min log-prob (drop already-easy examples)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1210,12 +1200,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-LOGPROB-FILTER</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-synthesis-e009</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-logprob-filter-e008</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1227,12 +1217,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-EVAL-chat-template-parity</t>
+          <t>TASK-E009-synthesis-kernel</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
+          <t>Synthesis: combine winning ablation choices into final config</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1240,21 +1230,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-synthesis-e009</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-fixture</t>
+          <t>TASK-EVAL-chat-template-parity</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
+          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1264,19 +1264,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-score-ingest</t>
+          <t>TASK-EVAL-cv-fixture</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
+          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1286,19 +1286,19 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-EVAL-cv-score-ingest</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
+          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1308,19 +1308,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-FIX-kernel-metadata</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1330,24 +1330,19 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-FIX-kernel-metadata</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1355,31 +1350,26 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
-        </is>
-      </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>US-OPS</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TASK-OPS-auto-rescue</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1387,70 +1377,80 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>H-OPS</t>
+        </is>
+      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-OPS-cron-trigger</t>
+          <t>TASK-OPS-auto-rescue</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
+          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(scheduler only)</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>US-meta</t>
+          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-OPS-gpu-dispatch-op</t>
+          <t>TASK-OPS-cron-trigger</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
+          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
+          <t>(scheduler only)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>US-meta</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-OPS-run-kernel-runner</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
+          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1460,149 +1460,139 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-OPS-run-kernel-runner</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>H-001</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-R1</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>H-001</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-R10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>H-006</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>US-4</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1612,12 +1602,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1629,93 +1619,93 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R11</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>H-007</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>US-1</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1730,7 +1720,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -1742,12 +1732,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1757,34 +1747,29 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1794,29 +1779,34 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1826,12 +1816,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1843,12 +1833,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1863,7 +1853,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1875,81 +1865,81 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>US-3</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1959,12 +1949,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -1976,12 +1966,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1991,12 +1981,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2008,12 +1998,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2023,12 +2013,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2040,12 +2030,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2055,29 +2045,29 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2087,29 +2077,29 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2119,12 +2109,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2136,12 +2126,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2151,12 +2141,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2168,12 +2158,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2183,12 +2173,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2200,12 +2190,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2215,29 +2205,29 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R29-eval-per-category-breakdown</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2252,29 +2242,24 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+          <t>US-2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2289,29 +2274,29 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
+          <t>TASK-R8</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>Local CV eval harness mirroring host scoring</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2326,81 +2311,184 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-2</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-gate-decision</t>
+          <t>TASK-R9</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-package-zip</t>
+          <t>TASK-RESEARCH-mine-discussions</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+          <t>Mine 200+ discussions for ranked actionable insights</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_insights_v1.md</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>TASK-RESEARCH-mine-top-notebooks</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Mine top 5 public NVIDIA Nemotron notebooks for techniques + write side-by-side comparison</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/top_notebooks_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>TASK-RESEARCH-winner-vs-ours</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Gap analysis: winner solution vs our current fork notebook</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_vs_current_v1.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-gate-decision</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-package-zip</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>TASK-SUBMIT-validate-adapter</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B67" t="inlineStr">
         <is>
           <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
         <is>
           <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
         </is>
@@ -2417,7 +2505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2936,12 +3024,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-PARALLEL-RESEARCH</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2951,24 +3039,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>~equal LB, 2x cheaper experiments</t>
+          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md, technique-backlog.md</t>
+          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2978,24 +3066,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>~equal LB at half cost; may slightly improve generalization.</t>
+          <t>~equal LB, 2x cheaper experiments</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>H-SUBMIT-GATE</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3005,24 +3093,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+          <t>~equal LB at half cost; may slightly improve generalization.</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-SUBMIT-GATE</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3032,37 +3120,64 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>+0.17 LB on 1594 unit_conversion rows</t>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>H-UNIT-CONV-100</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>+0.17 LB on 1594 unit_conversion rows</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>H-VLLM-EVAL</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>
@@ -3532,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3557,6 +3672,74 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>3423175478610363796</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TASK-DATA-cot-corpus-v1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4066723169138526005</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TASK-RESEARCH-winner-vs-ours</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>7816444016371433148</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TASK-RESEARCH-mine-discussions</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>8614860216596085950</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TASK-RESEARCH-mine-top-notebooks</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
CRITICAL: v15 smoke overwrote training code; restored v13 pipeline as v16 (4 cells, 4 dataSources, bindings preserved)
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T21:02:55.955233+00:00</t>
+          <t>2026-05-30T21:17:17.640735+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2491,6 +2491,94 @@
       <c r="E67" t="inlineStr">
         <is>
           <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-community-and-tabs</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Excel: community-sources + 6 analyses + 7 tab pages + technique-backlog into one workbook</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/community_and_tabs.xlsx, tests/test_community_and_tabs.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-discussions-extract</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Excel: structured extraction from all 217 discussion-*.md threads</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_extract.xlsx, tests/test_discussions_extract.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-master-roadmap</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Excel: master roadmap consolidating findings from the 3 other workbooks into a single shippable plan</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/master_roadmap.xlsx, tests/test_master_roadmap.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-winner-code-analysis</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Excel: per-file deep analysis of all 17 winner-* code files</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_code_analysis.xlsx, tests/test_winner_code_analysis.py</t>
         </is>
       </c>
     </row>
@@ -2505,7 +2593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2754,12 +2842,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-DEEP-ANALYSIS-XLSX</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
+          <t>Per-source markdown is hard to compare/rank. Structured Excel sheets with the same column vocabulary across sources (winner code, 217 discussions, community, tabs) make the operator's next-experiment decision provable: rank by (expected_cv_delta / effort), pick the top, push it.</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2769,24 +2857,24 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
+          <t>Decision quality. Replaces 'operator skim 1MB of markdown' with 'operator reads 5-sheet xlsx with ranked experiments + code-change pseudocode for each.'</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
+          <t>references/winner-*.md (17), references/discussion-*.md (217), references/community-sources.md, references/tab-*.md (7)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>H-EQ-FALLBACK</t>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Default to absolute-difference fallback in equation_numeric solvers when no rule is found; captures edge cases.</t>
+          <t>DATA QUALITY is the dominant lever: per-category deterministic solvers + verified oxed{} CoT corpora beat fancier training regimes.</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2796,24 +2884,24 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>+0.01 LB on equation_numeric category.</t>
+          <t>+0.20 LB (matches winner 0.85 vs naive baselines ~0.65)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-reasoning.py.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md, technique-backlog.md, winner-reasoning.py.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-EQ-FALLBACK</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Equation-numeric problems are solvable with SymPy linear/quadratic solvers; algebraic CoT is reproducible.</t>
+          <t>Default to absolute-difference fallback in equation_numeric solvers when no rule is found; captures edge cases.</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2823,24 +2911,24 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>+0.07 LB on equation_numeric_deduce(596)+_guess(136) categories</t>
+          <t>+0.01 LB on equation_numeric category.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, technique-backlog.md</t>
+          <t>analysis-discussions-deltas.md, winner-reasoning.py.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>H-GPU-DISPATCH</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
+          <t>Equation-numeric problems are solvable with SymPy linear/quadratic solvers; algebraic CoT is reproducible.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2850,24 +2938,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
+          <t>+0.07 LB on equation_numeric_deduce(596)+_guess(136) categories</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
+          <t>winner-reasoning.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-GPU-DISPATCH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
+          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2877,24 +2965,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
+          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
+          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2904,78 +2992,78 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+0.01 LB on hard categories.</t>
+          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-LOGPROB-FILTER</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>SUPPORTED</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>matches winner; cheaper variants underperform</t>
+          <t>+0.01 LB on hard categories.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md</t>
+          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>H-MAMBA-TARGETS</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Unblocks training on free GPU. Critical precondition.</t>
+          <t>matches winner; cheaper variants underperform</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, multiple discussions</t>
+          <t>winner-train_sft.py.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>H-NORL</t>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
+          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2985,24 +3073,24 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>saves compute; lower risk</t>
+          <t>Unblocks training on free GPU. Critical precondition.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md</t>
+          <t>analysis-discussions-deltas.md, multiple discussions</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-NORL</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
+          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3012,24 +3100,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>+0.16 LB on 1576 numeral rows</t>
+          <t>saves compute; lower risk</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H-PARALLEL-RESEARCH</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
+          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3039,24 +3127,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
+          <t>+0.16 LB on 1576 numeral rows</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-PARALLEL-RESEARCH</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3066,24 +3154,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>~equal LB, 2x cheaper experiments</t>
+          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md, technique-backlog.md</t>
+          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3093,24 +3181,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>~equal LB at half cost; may slightly improve generalization.</t>
+          <t>~equal LB, 2x cheaper experiments</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>H-SUBMIT-GATE</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3120,24 +3208,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+          <t>~equal LB at half cost; may slightly improve generalization.</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-SUBMIT-GATE</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3147,37 +3235,64 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>+0.17 LB on 1594 unit_conversion rows</t>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>H-UNIT-CONV-100</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>+0.17 LB on 1594 unit_conversion rows</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>H-VLLM-EVAL</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>
@@ -3647,7 +3762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3692,12 +3807,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4066723169138526005</t>
+          <t>3959759277942667967</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-winner-vs-ours</t>
+          <t>TASK-XLSX-community-and-tabs</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3709,12 +3824,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>7816444016371433148</t>
+          <t>4066723169138526005</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-mine-discussions</t>
+          <t>TASK-RESEARCH-winner-vs-ours</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3726,15 +3841,66 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>4245240514941347715</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-discussions-extract</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>7816444016371433148</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TASK-RESEARCH-mine-discussions</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>8614860216596085950</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>TASK-RESEARCH-mine-top-notebooks</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>QUEUED</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>9470450860965081304</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-winner-code-analysis</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
         <is>
           <t>QUEUED</t>
         </is>

</xml_diff>

<commit_message>
campaign CRON1: reconcile merged sessions + push notebook v43 (run-ready)
- Reconciled stale state: PRs #56/#59 already merged; cleared 2 sessions, tasks DONE
- Diagnosed recent 'COMPLETE' as QuickSave HTML render (no GPU execution)
- Audited live notebook v42, found+fixed 3 run-blocking gaps -> v43:
  * empty cell 0 -> restored nvidia-utility-script site.addsitedir bootstrap
    (cutlass.cute/Mamba3) + Blackwell ptxas /tmp mirror
  * stale eval cell overwrote cv_score.json -> replaced with submission.zip packaging
  * adapter now packaged (rank<=32 validated)
- New tool: tools/patch_notebook_bootstrap.py

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-30T21:27:53.438974+00:00</t>
+          <t>2026-05-31T02:53:29.027458+00:00</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -826,34 +826,34 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TASK-DATA-cot-corpus-v1</t>
+          <t>TASK-ABLATION-configs</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Build CoT corpus from train.csv using winner's deterministic solver pattern (the 0.65-&gt;0.85 lever)</t>
+          <t>Pre-build 5 ablation config JSONs (rank16, 2epoch, curriculum, select2reason, logprob_filter)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/, tests/test_cot_corpus_v1.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/ablation_configs.py, competitions/nvidia-nemotron-model-reasoning-challenge/experiments/README.md, tests/test_ablation_configs.py</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TASK-E-PRECOND-mamba-targets-smoke</t>
+          <t>TASK-CORPUS-scale-9cat</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Smoke-train kernel (10 steps) validating Mamba mixer LoRA targeting</t>
+          <t>Scale CoT corpus to 3K+ rows across ALL 9 host categories (winner-grade volume)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -861,31 +861,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>H-MAMBA-TARGETS</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/v4/, tests/test_corpus_v4_quality.py</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TASK-E001-corpus-v1</t>
+          <t>TASK-DATA-cot-corpus-v1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Assemble corpus.jsonl v1 from landed solvers (winner build_datum convention)</t>
+          <t>Build CoT corpus from train.csv using winner's deterministic solver pattern (the 0.65-&gt;0.85 lever)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -893,36 +883,31 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>H-DQ</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>US-3</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/, tests/test_cot_corpus_v1.py</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TASK-E002-SMOKE-RUN</t>
+          <t>TASK-E-PRECOND-mamba-targets-smoke</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Kaggle GPU smoke run: 5-min rank=4 max_steps=20 100-row preflight</t>
+          <t>Smoke-train kernel (10 steps) validating Mamba mixer LoRA targeting</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -939,12 +924,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TASK-E002-baseline-kernel</t>
+          <t>TASK-E001-corpus-v1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Finalize winner-faithful baseline training kernel (rank32/alpha64/1-epoch/LinearDecay)</t>
+          <t>Assemble corpus.jsonl v1 from landed solvers (winner build_datum convention)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -954,39 +939,39 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TASK-E002-push-and-train</t>
+          <t>TASK-E002-SMOKE-RUN</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Push baseline E-002 (rank=32) kernel to Kaggle GPU and ingest cv_score</t>
+          <t>Kaggle GPU smoke run: 5-min rank=4 max_steps=20 100-row preflight</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BLOCKED</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-smoke-mamba</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -998,12 +983,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TASK-E003-rank16-finalize</t>
+          <t>TASK-E002-baseline-kernel</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Align rank-16 ablation kernel (R24) with the E-002 config except rank/alpha</t>
+          <t>Finalize winner-faithful baseline training kernel (rank32/alpha64/1-epoch/LinearDecay)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1013,12 +998,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1030,27 +1015,22 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TASK-E004-2epoch-kernel</t>
+          <t>TASK-E002-push-and-train</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Clone baseline kernel with epochs=2 (refutation test for H-1EPOCH)</t>
+          <t>Push baseline E-002 (rank=32) kernel to Kaggle GPU and ingest cv_score</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>H-1EPOCH</t>
+          <t>BLOCKED</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-2epoch-e004</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-baseline-e002</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1062,12 +1042,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TASK-E005-curriculum-wire</t>
+          <t>TASK-E003-rank16-finalize</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Wire R23 curriculum config into the baseline kernel (difficulty-ascending)</t>
+          <t>Align rank-16 ablation kernel (R24) with the E-002 config except rank/alpha</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1077,12 +1057,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-curriculum-e005</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1094,12 +1074,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TASK-E006-select2reason</t>
+          <t>TASK-E004-2epoch-kernel</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Select2Reason curation: keep top-utility ~30 percent of corpus, then train baseline</t>
+          <t>Clone baseline kernel with epochs=2 (refutation test for H-1EPOCH)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1109,12 +1089,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-1EPOCH</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-select2reason-e006</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-2epoch-e004</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1126,12 +1106,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TASK-E007-RESCOPE</t>
+          <t>TASK-E005-curriculum-wire</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Rescope or abort stuck E-007 cryptarithm-guess Jules session</t>
+          <t>Wire R23 curriculum config into the baseline kernel (difficulty-ascending)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1139,26 +1119,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>H-CURRICULUM</t>
+        </is>
+      </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/v1, competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm, competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-curriculum-e005</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TASK-E007-cryptarithm-guess-integration</t>
+          <t>TASK-E006-select2reason</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Integrate cryptarithm_guess solver into corpus (winner skipped this category) — priority</t>
+          <t>Select2Reason curation: keep top-utility ~30 percent of corpus, then train baseline</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1168,29 +1153,29 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM-GUESS</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-select2reason-e006</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TASK-E008-logprob-filter</t>
+          <t>TASK-E007-RESCOPE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Pre-filter corpus by base-model min log-prob (drop already-easy examples)</t>
+          <t>Rescope or abort stuck E-007 cryptarithm-guess Jules session</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1198,31 +1183,26 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>H-LOGPROB-FILTER</t>
-        </is>
-      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-logprob-filter-e008</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/corpus/v1, competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm, competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TASK-E009-synthesis-kernel</t>
+          <t>TASK-E007-cryptarithm-guess-integration</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Synthesis: combine winning ablation choices into final config</t>
+          <t>Integrate cryptarithm_guess solver into corpus (winner skipped this category) — priority</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1232,29 +1212,29 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM-GUESS</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-synthesis-e009</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-e007-cryptarithm</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TASK-EVAL-chat-template-parity</t>
+          <t>TASK-E008-logprob-filter</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
+          <t>Pre-filter corpus by base-model min log-prob (drop already-easy examples)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1262,21 +1242,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>H-LOGPROB-FILTER</t>
+        </is>
+      </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-logprob-filter-e008</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-fixture</t>
+          <t>TASK-E009-synthesis-kernel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
+          <t>Synthesis: combine winning ablation choices into final config</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1284,21 +1274,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-synthesis-e009</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TASK-EVAL-cv-score-ingest</t>
+          <t>TASK-EVAL-chat-template-parity</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
+          <t>Add eval/chat_template_fixture.jsonl + tests/test_chat_template_parity.py asserting byte-equality vs official tokenizer</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1308,19 +1308,19 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/chat_template_fixture.jsonl, tests/test_chat_template_parity.py</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-EVAL-cv-fixture</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
+          <t>Build held-out CV fixture (200 rows stratified across 9 categories) for vllm_eval.py</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1330,19 +1330,19 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_build_cv_fixture.py</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TASK-FIX-kernel-metadata</t>
+          <t>TASK-EVAL-cv-fixture-9cat</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
+          <t>Build held-out CV fixture (300 rows stratified across all 9 host categories)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1352,24 +1352,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/cv_fixture_v2_manifest.json, competitions/nvidia-nemotron-model-reasoning-challenge/eval/build_cv_fixture_v2.py, competitions/nvidia-nemotron-model-reasoning-challenge/eval/README.md, tests/test_cv_fixture_v2.py</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-EVAL-cv-score-ingest</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Add record_cv_score state op + auto best_cv update + apply_decision pickup from kernel-output</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1377,31 +1372,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
-        </is>
-      </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>US-OPS</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, orchestrator/status.py, tests/test_record_cv_score.py</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-OPS-auto-rescue</t>
+          <t>TASK-EVAL-host-chat-template</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
+          <t>Capture exact Nemotron host chat template + reasoning_on system prompt for parity testing</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1411,46 +1396,41 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/host_template_spec.md, competitions/nvidia-nemotron-model-reasoning-challenge/eval/test_template_parity.py</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-OPS-cron-trigger</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(scheduler only)</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>US-meta</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-OPS-gpu-dispatch-op</t>
+          <t>TASK-FIX-kernel-metadata</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
+          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1460,19 +1440,24 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-OPS-run-kernel-runner</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1480,119 +1465,124 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>H-OPS</t>
+        </is>
+      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-NOTEBOOK-stratified-batching</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Add stratified-batching sampler tunable block to notebook (winner pattern, per-category mix)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>H-001</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/notebook_patches/v25_stratified.py, tests/test_stratified_batching.py</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-NOTEBOOK-target-masking</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Add target-masking + step-based LR decay tunable block to notebook (winner pattern)</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/notebook_patches/v24_target_masking.py, tests/test_notebook_patch_v24.py</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
+          <t>TASK-OPS-auto-rescue</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>H-006</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>US-4</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-OPS-cron-trigger</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
           <t>SUPERSEDED</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>(scheduler only)</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>US-meta</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1600,31 +1590,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>H-006</t>
-        </is>
-      </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
+          <t>TASK-OPS-run-kernel-runner</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1632,31 +1612,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>H-LORA32</t>
-        </is>
-      </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R1</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1666,12 +1636,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1681,14 +1651,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1700,76 +1670,61 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1779,34 +1734,29 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1816,130 +1766,110 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R11</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>US-1</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>H-001</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1949,29 +1879,29 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1981,29 +1911,34 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2013,29 +1948,29 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2045,29 +1980,29 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2077,61 +2012,66 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>US-3</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2141,12 +2081,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2158,12 +2098,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2173,12 +2113,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -2190,12 +2130,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2205,12 +2145,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2222,12 +2162,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2237,29 +2177,29 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2269,34 +2209,29 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2306,34 +2241,29 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>US-2</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2343,122 +2273,162 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-mine-discussions</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Mine 200+ discussions for ranked actionable insights</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_insights_v1.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-mine-top-notebooks</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Mine top 5 public NVIDIA Nemotron notebooks for techniques + write side-by-side comparison</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/top_notebooks_v1.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-winner-vs-ours</t>
+          <t>TASK-R29-eval-per-category-breakdown</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Gap analysis: winner solution vs our current fork notebook</t>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_vs_current_v1.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>US-2</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-gate-decision</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-package-zip</t>
+          <t>TASK-R8</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+          <t>Local CV eval harness mirroring host scoring</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2466,21 +2436,36 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-validate-adapter</t>
+          <t>TASK-R9</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2488,95 +2473,242 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TASK-XLSX-community-and-tabs</t>
+          <t>TASK-RESEARCH-mine-discussions</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Excel: community-sources + 6 analyses + 7 tab pages + technique-backlog into one workbook</t>
+          <t>Mine 200+ discussions for ranked actionable insights</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/community_and_tabs.xlsx, tests/test_community_and_tabs.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_insights_v1.md</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TASK-XLSX-discussions-extract</t>
+          <t>TASK-RESEARCH-mine-top-notebooks</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Excel: structured extraction from all 217 discussion-*.md threads</t>
+          <t>Mine top 5 public NVIDIA Nemotron notebooks for techniques + write side-by-side comparison</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_extract.xlsx, tests/test_discussions_extract.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/top_notebooks_v1.md</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TASK-XLSX-master-roadmap</t>
+          <t>TASK-RESEARCH-winner-vs-ours</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Excel: master roadmap consolidating findings from the 3 other workbooks into a single shippable plan</t>
+          <t>Gap analysis: winner solution vs our current fork notebook</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>BACKLOG</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/master_roadmap.xlsx, tests/test_master_roadmap.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_vs_current_v1.md</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>TASK-SUBMIT-gate-decision</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-package-zip</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>TASK-SUBMIT-validate-adapter</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-community-and-tabs</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Excel: community-sources + 6 analyses + 7 tab pages + technique-backlog into one workbook</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/community_and_tabs.xlsx, tests/test_community_and_tabs.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-discussions-extract</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Excel: structured extraction from all 217 discussion-*.md threads</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_extract.xlsx, tests/test_discussions_extract.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-master-roadmap</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Excel: master roadmap consolidating findings from the 3 other workbooks into a single shippable plan</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/master_roadmap.xlsx, tests/test_master_roadmap.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
           <t>TASK-XLSX-winner-code-analysis</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>Excel: per-file deep analysis of all 17 winner-* code files</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_code_analysis.xlsx, tests/test_winner_code_analysis.py</t>
         </is>
@@ -2593,7 +2725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2950,12 +3082,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>H-GPU-DISPATCH</t>
+          <t>H-FINAL-PREP-PARALLEL</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
+          <t>4 Jules workers (corpus-scale 9cat, cv-fixture 9cat, host-template-parity, ablation-configs) + operator-side notebook v23 (chat template + reasoning_on + full corpus) + corpus-uploader tool close all 10 gaps from the readiness audit in parallel; once landed, the operator can run baseline + 5 ablations within 3 days.</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2965,24 +3097,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
+          <t>From 'pipeline-validation' state to 'final-quality-runnable' state within 24h.</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
+          <t>readiness audit (10 gaps), ROADMAP.md, references/analysis-winner-training-internals.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-GPU-DISPATCH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
+          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2992,24 +3124,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
+          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
+          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3019,78 +3151,78 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+0.01 LB on hard categories.</t>
+          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-LOGPROB-FILTER</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>SUPPORTED</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>matches winner; cheaper variants underperform</t>
+          <t>+0.01 LB on hard categories.</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md</t>
+          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>H-MAMBA-TARGETS</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Unblocks training on free GPU. Critical precondition.</t>
+          <t>matches winner; cheaper variants underperform</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, multiple discussions</t>
+          <t>winner-train_sft.py.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>H-NORL</t>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
+          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -3100,24 +3232,24 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>saves compute; lower risk</t>
+          <t>Unblocks training on free GPU. Critical precondition.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md</t>
+          <t>analysis-discussions-deltas.md, multiple discussions</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-NORL</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
+          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3127,24 +3259,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>+0.16 LB on 1576 numeral rows</t>
+          <t>saves compute; lower risk</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>H-PARALLEL-RESEARCH</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
+          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3154,24 +3286,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
+          <t>+0.16 LB on 1576 numeral rows</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-PARALLEL-RESEARCH</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3181,24 +3313,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>~equal LB, 2x cheaper experiments</t>
+          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md, technique-backlog.md</t>
+          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3208,24 +3340,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>~equal LB at half cost; may slightly improve generalization.</t>
+          <t>~equal LB, 2x cheaper experiments</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>H-SUBMIT-GATE</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3235,24 +3367,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+          <t>~equal LB at half cost; may slightly improve generalization.</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-SUBMIT-GATE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3262,37 +3394,64 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>+0.17 LB on 1594 unit_conversion rows</t>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>H-UNIT-CONV-100</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>+0.17 LB on 1594 unit_conversion rows</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>H-VLLM-EVAL</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>
@@ -3762,7 +3921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3787,125 +3946,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>3423175478610363796</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>TASK-DATA-cot-corpus-v1</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>3959759277942667967</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>TASK-XLSX-community-and-tabs</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>4066723169138526005</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>TASK-RESEARCH-winner-vs-ours</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>4245240514941347715</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>TASK-XLSX-discussions-extract</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>7816444016371433148</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>TASK-RESEARCH-mine-discussions</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>8614860216596085950</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>TASK-RESEARCH-mine-top-notebooks</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>9470450860965081304</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>TASK-XLSX-winner-code-analysis</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>QUEUED</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
campaign CRON3: host-faithful CV gen params -> notebook v45
Verified vs OFFICIAL Evaluation page:
- submission format CONFIRMED: submission.zip (LoRA adapter, rank<=32, adapter_config.json) -- v44 packaging correct
- gen-param contradiction RESOLVED: host scores temp=0.0(greedy)/max_tokens=7680/max_model_len=8192
  via vLLM, NOT the winner-notebook evaluate() defaults (1.0/3584/4096) our spec had
- patched notebook cell 2 -> v45; corrected eval/host_template_spec.md
- ledger: +C-GENPARAMS-RESOLVED decision, +H-GENPARITY hypothesis

Key fix: temp 1.0->0.0. Host decodes greedily, so a sampling-based CV never predicted the LB.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-31T02:53:29.027458+00:00</t>
+          <t>2026-05-31T07:43:53.550905+00:00</t>
         </is>
       </c>
     </row>
@@ -503,7 +503,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -2725,7 +2725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3109,12 +3109,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>H-GPU-DISPATCH</t>
+          <t>H-GENPARITY</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
+          <t>Evaluating local CV with host-exact gen params (temp=0.0 greedy, max_tokens=7680, max_model_len=8192) yields a CV that tracks the leaderboard within a small constant offset; sampling-based CV (temp=1.0) does not.</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3124,24 +3124,24 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
+          <t>CV becomes a reliable submit gate; reduces wasted submissions on CV that doesn't transfer.</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
+          <t>official Evaluation page 2026-05-31, eval/host_template_spec.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-GPU-DISPATCH</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
+          <t>Today the loop stops at 'kernel authored by Jules and merged to main' - the actual Kaggle GPU run is a manual operator action. Adding a gpu_dispatch ledger op + a tools/run_kernel.py runner (kernel-push -&gt; poll kernel-status -&gt; kernel-output) lets the operator's owner-role automatically promote a merged experiment with status=READY_FOR_GPU into a live Kaggle kernel run and capture cv_score.json + adapter dir into the ledger, completing the train-&gt;validate loop.</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -3151,24 +3151,24 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
+          <t>Removes the only manual hand-off in the loop; enables the operator's 30-min cron to also drive Kaggle GPU runs autonomously; unlocks the full E-002 -&gt; E-003..E-009 ablation fanout to run end-to-end.</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md kernel-experiment pattern, tools/kaggle_lite.py kernel-push/kernel-status/kernel-output, orchestrator/loop.py poll_in_flight</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>H-LOGPROB-FILTER</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
+          <t>Gravity-category problems (free-fall/projectile/orbital mechanics) reduce to closed-form physics formulas and admit a deterministic solver.</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -3178,78 +3178,78 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>+0.01 LB on hard categories.</t>
+          <t>+0.17 LB from solving all 1597 gravity rows (16.8% of train)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>H-LORA32</t>
+          <t>H-LOGPROB-FILTER</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
+          <t>Filtering out examples whose base-model min-logprob &gt; -0.05 prevents over-tuning on easy examples and improves accuracy on hard rules.</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SUPPORTED</t>
+          <t>PROPOSED</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>matches winner; cheaper variants underperform</t>
+          <t>+0.01 LB on hard categories.</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md</t>
+          <t>analysis-discussions-deltas.md, winner-loss_config.py.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>H-MAMBA-TARGETS</t>
+          <t>H-LORA32</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
+          <t>LoRA rank 32 / alpha 64 SFT (winner config) is the right anchor; deviations should justify themselves with CV evidence.</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>PROPOSED</t>
+          <t>SUPPORTED</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Unblocks training on free GPU. Critical precondition.</t>
+          <t>matches winner; cheaper variants underperform</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, multiple discussions</t>
+          <t>winner-train_sft.py.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>H-NORL</t>
+          <t>H-MAMBA-TARGETS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
+          <t>Explicit Mamba mixer LoRA targeting (mixer.in_proj, mixer.out_proj) + attention-only avoids the MoE expert-scan hang and enables training on 2xT4 4-bit.</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3259,24 +3259,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>saves compute; lower risk</t>
+          <t>Unblocks training on free GPU. Critical precondition.</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>winner-INDEX.md, DIGEST-community.md</t>
+          <t>analysis-discussions-deltas.md, multiple discussions</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-NORL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
+          <t>RL / distillation are NOT needed; pure SFT on verified CoT reaches top-LB.</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3286,24 +3286,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>+0.16 LB on 1576 numeral rows</t>
+          <t>saves compute; lower risk</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>winner-INDEX.md, DIGEST-community.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>H-PARALLEL-RESEARCH</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
+          <t>Numeral-system problems (base conversions, radix arithmetic, novel digit systems) are deterministic given the rules in the prompt.</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3313,24 +3313,24 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
+          <t>+0.16 LB on 1576 numeral rows</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-PARALLEL-RESEARCH</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
+          <t>While the GPU iteration is single-threaded (we wait on browser Save&amp;Run All), 4 parallel Jules sessions can mine top notebooks, dig through 200+ discussions, synthesize CoT corpus, and gap-analyze vs winner — all CPU-only, all producing concrete analysis/data files the operator reads on next cycle to inform the next code push and the next training experiment.</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3340,24 +3340,24 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>~equal LB, 2x cheaper experiments</t>
+          <t>Decouples campaign throughput from the GPU bottleneck. Each research task produces a concrete file that influences the next code push. Most impactful: the CoT corpus (winner's 0.65-&gt;0.85 lever).</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>winner-train_sft.py.md, technique-backlog.md</t>
+          <t>references/technique-backlog.md, references/analysis-winner.md, 210 discussion-*.md files</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>H-SELECT2REASON</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
+          <t>LoRA rank 16 (half the cap) reaches within 0.005 of rank-32 with half the parameters; ablation worth running for compute efficiency.</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3367,24 +3367,24 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>~equal LB at half cost; may slightly improve generalization.</t>
+          <t>~equal LB, 2x cheaper experiments</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
+          <t>winner-train_sft.py.md, technique-backlog.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>H-SUBMIT-GATE</t>
+          <t>H-SELECT2REASON</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
+          <t>Select2Reason-style curation (drop low-utility / repetitive traces) matches baseline accuracy at ~30 percent of cost.</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3394,24 +3394,24 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
+          <t>~equal LB at half cost; may slightly improve generalization.</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
+          <t>analysis-discussions-deltas.md, konbu17 discussion</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-SUBMIT-GATE</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+          <t>A tools/validate_adapter.py that (a) loads base+adapter via peft, (b) asserts the adapter_config rank &lt;= 32, (c) runs 5 sample prompts through the adapter and confirms each output contains \boxed{...}, and (d) returns 0 only on full pass - used as a precondition by both the dispatcher submission_proposal flow and the operator submit gate - eliminates wasted submits on adapters that fail to load, exceed rank, or omit the required answer format.</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3421,37 +3421,64 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>+0.17 LB on 1594 unit_conversion rows</t>
+          <t>Saves &gt;=1 wasted submit/day in practice (real cap is 5/day, 2 reserved finals); makes the unsupervised auto-merge safer because broken-adapter PRs cannot accidentally trigger a submit.</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+          <t>AGENTS.md submission handoff, tools/kaggle_lite.py submission-upload</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>H-UNIT-CONV-100</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Unit-conversion problems decompose into a directed graph of conversion factors; a Floyd-Warshall closure over the parsed factors yields exact answers.</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PROPOSED</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>+0.17 LB on 1594 unit_conversion rows</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>winner-reasoning.py.md, data/taxonomy/taxonomy.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>H-VLLM-EVAL</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>Building eval/vllm_eval.py that loads (base + adapter), runs inference with temperature=0.0/top_p=1.0/max_tokens=7680/max_model_len=8192/max_lora_rank=32 and extracts \boxed{...} for exact (and +/-1e-2 numeric) match against a held-out CV slice gives us a reproducible local CV metric that the operator-side submit gate can compare against best_cv, preventing burned submit slots on duplicates and surfacing regressions before they hit the leaderboard.</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>PROPOSED</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Per technique-backlog #2 (effort:M, expected_gain:HIGH); enables every other iteration and prevents wasted submits against the 5/day hard cap; mirrors winner dashboards.</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>technique-backlog.md #2, analysis-winner-training-internals.md, winner-train_sft.py.md</t>
         </is>
@@ -3820,7 +3847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3843,32 +3870,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>D-AUDIT-2026-05-30</t>
+          <t>C-GENPARAMS-RESOLVED</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Pause new feature work; land the 6 audit-corrections + 5 seeded tasks before adding capability.</t>
+          <t>Adopt the OFFICIAL Evaluation page gen params as authoritative for local CV: temperature=0.0 (greedy), max_tokens=7680, top_p=1.0, max_model_len=8192, max_lora_rank=32. Winner-notebook evaluate() defaults (1.0/3584/4096) are NON-authoritative.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Audit found 5 live defects (3 fixed mid-pass), 6 invalidated assumptions, 0 end-to-end runs. Infrastructure-complete but execution-untriggered. Adding features now compounds cross-PR invariant drift the audit identified.</t>
+          <t>Host scores greedily; a CV measured at temp=1.0 sampling does not predict the leaderboard. temp 1.0-&gt;0.0 is the key fix.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>D-AUDIT-2026-05-30</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Pause new feature work; land the 6 audit-corrections + 5 seeded tasks before adding capability.</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Audit found 5 live defects (3 fixed mid-pass), 6 invalidated assumptions, 0 end-to-end runs. Infrastructure-complete but execution-untriggered. Adding features now compounds cross-PR invariant drift the audit identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>D-EXPLAN-001</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Lock experimentation plan (Phase A done, B-&gt;C-&gt;D-&gt;E-&gt;F; E-007 cryptarithm_guess prioritized).</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Cross-validated against winner repo (R13), discussion deltas (R11b), 18 ledger hypotheses. See EXPERIMENTATION_PLAN.md.</t>
         </is>

</xml_diff>

<commit_message>
campaign CRON4: hold v45 for baseline; queue 2 post-baseline eval improvements
GPU monitor: no fresh run (user not yet re-run v45); best_cv still None.
Disciplined hold: stop changing the notebook the user is about to run.
Planner: queued TASK-EVAL-percat-cv + TASK-EVAL-honest-dev-split (gated on baseline).
Pacing ~20min to avoid busy-looping on an external (user) GPU run.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/state/dashboard.xlsx
+++ b/state/dashboard.xlsx
@@ -455,7 +455,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-31T07:43:53.550905+00:00</t>
+          <t>2026-05-31T07:48:07.171348+00:00</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8">
@@ -527,7 +527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G77"/>
+  <dimension ref="A1:G79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1381,34 +1381,34 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TASK-EVAL-host-chat-template</t>
+          <t>TASK-EVAL-honest-dev-split</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Capture exact Nemotron host chat template + reasoning_on system prompt for parity testing</t>
+          <t>Hold out stratified dev set for honest CV gate</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/host_template_spec.md, competitions/nvidia-nemotron-model-reasoning-challenge/eval/test_template_parity.py</t>
+          <t>notebook cell 2/3</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TASK-EVAL-vllm-harness-skeleton</t>
+          <t>TASK-EVAL-host-chat-template</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
+          <t>Capture exact Nemotron host chat template + reasoning_on system prompt for parity testing</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1418,46 +1418,41 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/host_template_spec.md, competitions/nvidia-nemotron-model-reasoning-challenge/eval/test_template_parity.py</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TASK-FIX-kernel-metadata</t>
+          <t>TASK-EVAL-percat-cv</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
+          <t>Per-category stratified CV in eval cell</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>BACKLOG</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>notebook cell 1/2/3</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TASK-K0-kaggle-access-smoke</t>
+          <t>TASK-EVAL-vllm-harness-skeleton</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Kaggle access smoke test from the Jules VM</t>
+          <t>Write eval/vllm_eval.py harness skeleton with host-faithful params + \boxed{} extractor + per-category scoring</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1465,31 +1460,21 @@
           <t>DONE</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>H-OPS</t>
-        </is>
-      </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>US-OPS</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval/, tests/test_vllm_eval.py</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TASK-NOTEBOOK-stratified-batching</t>
+          <t>TASK-FIX-kernel-metadata</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Add stratified-batching sampler tunable block to notebook (winner pattern, per-category mix)</t>
+          <t>Replace TODO dataset_sources + model_sources in 8 kernel-metadata.json files</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1499,19 +1484,24 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/notebook_patches/v25_stratified.py, tests/test_stratified_batching.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TASK-NOTEBOOK-target-masking</t>
+          <t>TASK-K0-kaggle-access-smoke</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Add target-masking + step-based LR decay tunable block to notebook (winner pattern)</t>
+          <t>Kaggle access smoke test from the Jules VM</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1519,21 +1509,31 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>H-OPS</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/notebook_patches/v24_target_masking.py, tests/test_notebook_patch_v24.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/kaggle-access-smoke.md</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>US-OPS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TASK-OPS-auto-rescue</t>
+          <t>TASK-NOTEBOOK-stratified-batching</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
+          <t>Add stratified-batching sampler tunable block to notebook (winner pattern, per-category mix)</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1543,46 +1543,41 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/notebook_patches/v25_stratified.py, tests/test_stratified_batching.py</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TASK-OPS-cron-trigger</t>
+          <t>TASK-NOTEBOOK-target-masking</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
+          <t>Add target-masking + step-based LR decay tunable block to notebook (winner pattern)</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(scheduler only)</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>US-meta</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/experiments/notebook_patches/v24_target_masking.py, tests/test_notebook_patch_v24.py</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TASK-OPS-gpu-dispatch-op</t>
+          <t>TASK-OPS-auto-rescue</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
+          <t>Add auto-rescue path to poll_in_flight (COMPLETED-without-PR -&gt; extract patch + pytest + merge)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1592,90 +1587,90 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
+          <t>orchestrator/loop.py, orchestrator/github_ops.py, tests/test_auto_rescue.py</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TASK-OPS-run-kernel-runner</t>
+          <t>TASK-OPS-cron-trigger</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
+          <t>Schedule the autonomous operator tick (cron / Task Scheduler) - user approval</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
+          <t>(scheduler only)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>US-meta</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TASK-R1</t>
+          <t>TASK-OPS-gpu-dispatch-op</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Derive the problem-category taxonomy + classifier</t>
+          <t>Wire gpu_dispatch op into orchestrator/loop.py + state.py (auto-run merged kernels)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>H-001</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
+          <t>orchestrator/state.py, orchestrator/loop.py, tests/test_gpu_dispatch.py</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TASK-R1-category-taxonomy</t>
+          <t>TASK-OPS-run-kernel-runner</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Write tools/run_kernel.py end-to-end runner (kernel-push -&gt; poll status -&gt; pull outputs)</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>tools/run_kernel.py, tests/test_run_kernel.py</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TASK-R10</t>
+          <t>TASK-R1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
+          <t>Derive the problem-category taxonomy + classifier</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1685,29 +1680,29 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-1</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R1-category-taxonomy.md</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TASK-R10-sft-training-kernel</t>
+          <t>TASK-R1-category-taxonomy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1719,17 +1714,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TASK-R10a-train-script-and-smoke</t>
+          <t>TASK-R10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
+          <t>Author the QLoRA SFT training kernel (GPU-ready; runs later)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1739,110 +1734,110 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>US-4</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R10-sft-training-kernel.md</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TASK-R10b-kernel-metadata-readme</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
+          <t>TASK-R10-sft-training-kernel</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>H-LORA32</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>US-4</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TASK-R11</t>
+          <t>TASK-R10a-train-script-and-smoke</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Meta-analysis of the 217 discussion threads</t>
+          <t>QLoRA train.py + --smoke offline test (rank&lt;=32/alpha 64 asserted)</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>H-007</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/train.py</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>US-1</t>
-        </is>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TASK-R11-discussion-meta-analysis</t>
+          <t>TASK-R10b-kernel-metadata-readme</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Kaggle kernel-metadata.json + README for the training kernel</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>H-LORA32</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train/(kernel-metadata.json|README.md)</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TASK-R11a-discussion-do-avoid</t>
+          <t>TASK-R11</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
+          <t>Meta-analysis of the 217 discussion threads</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1852,56 +1847,41 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions.md</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>US-1</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R11-discussion-meta-analysis.md</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TASK-R11b-deltas-and-new-hypotheses</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
+          <t>TASK-R11-discussion-meta-analysis</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>H-007</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>US-1</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TASK-R12</t>
+          <t>TASK-R11a-discussion-do-avoid</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Public notebook + writeup skeleton (prize eligibility)</t>
+          <t>217 discussions → ranked Do / Avoid digest (cited)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1911,34 +1891,29 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>H-008</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-do-avoid.md</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>US-6</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TASK-R13-winner-trio-digest</t>
+          <t>TASK-R11b-deltas-and-new-hypotheses</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
+          <t>Deltas vs winner + ≥5 new hypotheses for the ledger</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1948,12 +1923,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>H-006</t>
+          <t>H-007</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-discussions-deltas.md</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -1965,12 +1940,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TASK-R1a-category-taxonomy-doc</t>
+          <t>TASK-R12</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Category taxonomy + value ranking (doc only)</t>
+          <t>Public notebook + writeup skeleton (prize eligibility)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -1980,29 +1955,34 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-008</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/writeup</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>US-1</t>
+          <t>US-6</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R12-writeup-skeleton.md</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TASK-R1b-category-classifier</t>
+          <t>TASK-R13-winner-trio-digest</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Rule classifier + tests for the taxonomy</t>
+          <t>Trio digest: winner LR schedule + loss config + train_common (clubbed)</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2012,12 +1992,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>H-001</t>
+          <t>H-006</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/references/analysis-winner-training-internals.md</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -2029,49 +2009,44 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TASK-R2.&lt;cat&gt;</t>
+          <t>TASK-R1a-category-taxonomy-doc</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
+          <t>Category taxonomy + value ranking (doc only)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>SUPERSEDED</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>H-002</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/taxonomy.md</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>US-3</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TASK-R20-cipher-solver</t>
+          <t>TASK-R1b-category-classifier</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
+          <t>Rule classifier + tests for the taxonomy</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2081,61 +2056,66 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>H-CIPHER-100</t>
+          <t>H-001</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/taxonomy/classify.py</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-1</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TASK-R21-equation-sympy-solver</t>
+          <t>TASK-R2.&lt;cat&gt;</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Equation-numeric SymPy solver + verification on holdout</t>
+          <t>Per-category deterministic solver  (TEMPLATE — operator clones one per category)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>SUPERSEDED</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>H-EQ-SYMPY</t>
+          <t>H-002</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/&lt;category&gt;</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>US-3</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R2-solver-template.md</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TASK-R22-bit-manipulation-solver</t>
+          <t>TASK-R20-cipher-solver</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
+          <t>Cipher-category deterministic solver + 100-sample holdout validation</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2145,12 +2125,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>H-BIT-NICKNAME</t>
+          <t>H-CIPHER-100</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cipher</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2162,12 +2142,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TASK-R23-curriculum-config</t>
+          <t>TASK-R21-equation-sympy-solver</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
+          <t>Equation-numeric SymPy solver + verification on holdout</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2177,12 +2157,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>H-CURRICULUM</t>
+          <t>H-EQ-SYMPY</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/equation_numeric</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2194,12 +2174,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TASK-R24-rank16-ablation-kernel</t>
+          <t>TASK-R22-bit-manipulation-solver</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
+          <t>Bit-manipulation deterministic solver via nickname regex extraction</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -2209,29 +2189,29 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>H-RANK16</t>
+          <t>H-BIT-NICKNAME</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/bit_manipulation</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>US-4</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TASK-R25-gravity-solver</t>
+          <t>TASK-R23-curriculum-config</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
+          <t>Difficulty estimator + curriculum-shuffle SFT config</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2241,12 +2221,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>H-GRAVITY-100</t>
+          <t>H-CURRICULUM</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation/curriculum.py</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2258,12 +2238,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TASK-R26-numeral-solver</t>
+          <t>TASK-R24-rank16-ablation-kernel</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
+          <t>Rank-16 LoRA ablation: kernel-metadata variant + smoke test</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2273,29 +2253,29 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>H-NUMERAL-100</t>
+          <t>H-RANK16</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/kernels/train-rank16</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>US-3</t>
+          <t>US-4</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TASK-R27-unit-conversion-solver</t>
+          <t>TASK-R25-gravity-solver</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
+          <t>Gravity-category deterministic solver (closed-form mechanics) + 100-sample validation</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2305,12 +2285,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>H-UNIT-CONV-100</t>
+          <t>H-GRAVITY-100</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/gravity</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2322,12 +2302,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TASK-R28-cryptarithm-solver</t>
+          <t>TASK-R26-numeral-solver</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
+          <t>Numeral-system deterministic solver (arbitrary radix + novel digit systems)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2337,12 +2317,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>H-CRYPTARITHM</t>
+          <t>H-NUMERAL-100</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/numeral</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2354,12 +2334,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>TASK-R29-eval-per-category-breakdown</t>
+          <t>TASK-R27-unit-conversion-solver</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Extend CV harness to report per-category accuracy + stratified split</t>
+          <t>Unit-conversion deterministic solver via Floyd-Warshall conversion graph</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2369,29 +2349,29 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-UNIT-CONV-100</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/unit_conversion</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>US-2</t>
+          <t>US-3</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>TASK-R7</t>
+          <t>TASK-R28-cryptarithm-solver</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Verified `\boxed{}` chain-of-thought generator</t>
+          <t>Cryptarithm-deduce solver via constraint propagation (python-constraint / Z3)</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2401,34 +2381,29 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>H-DQ</t>
+          <t>H-CRYPTARITHM</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/solvers/cryptarithm</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>US-3</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TASK-R8</t>
+          <t>TASK-R29-eval-per-category-breakdown</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Local CV eval harness mirroring host scoring</t>
+          <t>Extend CV harness to report per-category accuracy + stratified split</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2449,23 +2424,18 @@
       <c r="F66" t="inlineStr">
         <is>
           <t>US-2</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TASK-R9</t>
+          <t>TASK-R7</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Corpus curation: filter, dedup, difficulty-balance</t>
+          <t>Verified `\boxed{}` chain-of-thought generator</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2480,7 +2450,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/cot</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2490,19 +2460,19 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R7-cot-generator.md</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-mine-discussions</t>
+          <t>TASK-R8</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Mine 200+ discussions for ranked actionable insights</t>
+          <t>Local CV eval harness mirroring host scoring</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2510,21 +2480,36 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_insights_v1.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/eval</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>US-2</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R8-cv-harness.md</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-mine-top-notebooks</t>
+          <t>TASK-R9</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Mine top 5 public NVIDIA Nemotron notebooks for techniques + write side-by-side comparison</t>
+          <t>Corpus curation: filter, dedup, difficulty-balance</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2532,21 +2517,36 @@
           <t>DONE</t>
         </is>
       </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>H-DQ</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/top_notebooks_v1.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/data/curation</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>US-3</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>competitions\nvidia-nemotron-model-reasoning-challenge\tasks\todo\TASK-R9-corpus-curation.md</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TASK-RESEARCH-winner-vs-ours</t>
+          <t>TASK-RESEARCH-mine-discussions</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Gap analysis: winner solution vs our current fork notebook</t>
+          <t>Mine 200+ discussions for ranked actionable insights</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2556,41 +2556,41 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_vs_current_v1.md</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_insights_v1.md</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-gate-decision</t>
+          <t>TASK-RESEARCH-mine-top-notebooks</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
+          <t>Mine top 5 public NVIDIA Nemotron notebooks for techniques + write side-by-side comparison</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>IN_PROGRESS</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/top_notebooks_v1.md</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-package-zip</t>
+          <t>TASK-RESEARCH-winner-vs-ours</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
+          <t>Gap analysis: winner solution vs our current fork notebook</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2600,41 +2600,41 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>tools/package_submission.py, tests/test_package_submission.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_vs_current_v1.md</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>TASK-SUBMIT-validate-adapter</t>
+          <t>TASK-SUBMIT-gate-decision</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
+          <t>Add submit_decision step to orchestrator/loop.py (cv-beats-best + cap-headroom + ≤3/day gating)</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>DONE</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
+          <t>orchestrator/submit_gate.py, orchestrator/loop.py, tests/test_submit_gate.py</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TASK-XLSX-community-and-tabs</t>
+          <t>TASK-SUBMIT-package-zip</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Excel: community-sources + 6 analyses + 7 tab pages + technique-backlog into one workbook</t>
+          <t>Write tools/package_submission.py that builds submission.zip from an adapter dir (Kaggle format)</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2644,19 +2644,19 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/community_and_tabs.xlsx, tests/test_community_and_tabs.py</t>
+          <t>tools/package_submission.py, tests/test_package_submission.py</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TASK-XLSX-discussions-extract</t>
+          <t>TASK-SUBMIT-validate-adapter</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Excel: structured extraction from all 217 discussion-*.md threads</t>
+          <t>Write tools/validate_adapter.py pre-submit gate (loadability + rank&lt;=32 + boxed-output smoke)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2666,19 +2666,19 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_extract.xlsx, tests/test_discussions_extract.py</t>
+          <t>tools/validate_adapter.py, tests/test_validate_adapter.py</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TASK-XLSX-master-roadmap</t>
+          <t>TASK-XLSX-community-and-tabs</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Excel: master roadmap consolidating findings from the 3 other workbooks into a single shippable plan</t>
+          <t>Excel: community-sources + 6 analyses + 7 tab pages + technique-backlog into one workbook</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2688,27 +2688,71 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/master_roadmap.xlsx, tests/test_master_roadmap.py</t>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/community_and_tabs.xlsx, tests/test_community_and_tabs.py</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>TASK-XLSX-discussions-extract</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Excel: structured extraction from all 217 discussion-*.md threads</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/discussions_extract.xlsx, tests/test_discussions_extract.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>TASK-XLSX-master-roadmap</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Excel: master roadmap consolidating findings from the 3 other workbooks into a single shippable plan</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/master_roadmap.xlsx, tests/test_master_roadmap.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
           <t>TASK-XLSX-winner-code-analysis</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Excel: per-file deep analysis of all 17 winner-* code files</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>DONE</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
         <is>
           <t>competitions/nvidia-nemotron-model-reasoning-challenge/analysis/winner_code_analysis.xlsx, tests/test_winner_code_analysis.py</t>
         </is>

</xml_diff>